<commit_message>
Update general courses and class list
</commit_message>
<xml_diff>
--- a/pangaocal-main/通识课程数据库.xlsx
+++ b/pangaocal-main/通识课程数据库.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F276"/>
+  <dimension ref="A1:F278"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8698,6 +8698,66 @@
       <c r="F276" t="inlineStr">
         <is>
           <t>历史与文明</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>276</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>海洋与大气学院</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>海洋的前世今生</t>
+        </is>
+      </c>
+      <c r="D277" t="n">
+        <v>2</v>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>科学进步与科技创新</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>科学与技术</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>277</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>马克思主义学院</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>大学生爱国教育十讲</t>
+        </is>
+      </c>
+      <c r="D278" t="n">
+        <v>2</v>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>当代社会与公民责任</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>社会与文化</t>
         </is>
       </c>
     </row>
@@ -8712,7 +8772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F82"/>
+  <dimension ref="A1:F83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11172,6 +11232,36 @@
         </is>
       </c>
       <c r="F82" t="inlineStr">
+        <is>
+          <t>社会与文化</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>277</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>马克思主义学院</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>大学生爱国教育十讲</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>2</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>当代社会与公民责任</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
         <is>
           <t>社会与文化</t>
         </is>
@@ -14264,7 +14354,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F94"/>
+  <dimension ref="A1:F95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17089,6 +17179,36 @@
         </is>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>276</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>海洋与大气学院</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>海洋的前世今生</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>2</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>科学进步与科技创新</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>科学与技术</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add marine ecological disasters course
</commit_message>
<xml_diff>
--- a/pangaocal-main/通识课程数据库.xlsx
+++ b/pangaocal-main/通识课程数据库.xlsx
@@ -416,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F278"/>
+  <dimension ref="A1:F279"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8758,6 +8758,36 @@
       <c r="F278" t="inlineStr">
         <is>
           <t>社会与文化</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>278</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>环境科学与工程学院</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>漫话海洋生态灾害</t>
+        </is>
+      </c>
+      <c r="D279" t="n">
+        <v>2</v>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>科学进步与科技创新</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>科学与技术</t>
         </is>
       </c>
     </row>
@@ -14354,7 +14384,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F95"/>
+  <dimension ref="A1:F96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17209,6 +17239,36 @@
         </is>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>278</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>环境科学与工程学院</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>漫话海洋生态灾害</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>2</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>科学进步与科技创新</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>科学与技术</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>